<commit_message>
Changes for data understanding phases. Better graphs and tables
</commit_message>
<xml_diff>
--- a/docs/Data Understanding.xlsx
+++ b/docs/Data Understanding.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jkulinz-my.sharepoint.com/personal/k11717394_students_jku_at/Documents/Masterarbeit/PythonWorkspace/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chrig\PycharmProjects\PerturbationThesis\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="404" documentId="11_AD4DB114E441178AC67DF424E615FED4683EDF23" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{451BC326-43E5-4D03-B1D6-FC640FE3C6FC}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC5EF856-195E-4EE4-9D94-D9FF065070C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-75" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_FlightData" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="114">
   <si>
     <t>Flight Data</t>
   </si>
@@ -365,6 +365,9 @@
   </si>
   <si>
     <t>Find #flights landing one hour before each flight. Feature name: "PREF_FLIGHTS_1H"</t>
+  </si>
+  <si>
+    <t>Link: https://www.transtats.bts.gov/DatabaseInfo.asp?QO_VQ=EFD%20&amp;Yv0x=D</t>
   </si>
 </sst>
 </file>
@@ -374,7 +377,7 @@
   <numFmts count="1">
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -413,6 +416,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -515,32 +526,23 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -552,33 +554,26 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -586,21 +581,37 @@
     <xf numFmtId="41" fontId="0" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Dezimal [0]" xfId="1" builtinId="6"/>
+    <cellStyle name="Link" xfId="2" builtinId="8"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -896,88 +907,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
       <c r="F1" s="1"/>
     </row>
-    <row r="2" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-    </row>
-    <row r="3" spans="1:13" s="7" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-    </row>
-    <row r="4" spans="1:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:13" s="3" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="F4" s="23"/>
-      <c r="G4" s="8" t="s">
+      <c r="F4" s="12"/>
+      <c r="G4" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="H4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="I4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="J4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="K4" s="8" t="s">
+      <c r="K4" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="L4" s="8" t="s">
+      <c r="L4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="M4" s="8" t="s">
+      <c r="M4" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:13" s="7" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
+    <row r="5" spans="1:13" s="3" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="B5" s="24">
+      <c r="B5" s="17">
         <v>11292279</v>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="19">
         <v>29</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="27" t="s">
         <v>44</v>
       </c>
       <c r="E5" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="F5" s="18"/>
-      <c r="G5" s="21">
+      <c r="F5" s="10"/>
+      <c r="G5" s="11">
         <v>1</v>
       </c>
       <c r="H5" t="s">
@@ -986,13 +997,13 @@
       <c r="I5" t="s">
         <v>35</v>
       </c>
-      <c r="J5" s="9" t="s">
+      <c r="J5" s="5" t="s">
         <v>51</v>
       </c>
       <c r="K5">
         <v>748848</v>
       </c>
-      <c r="L5" s="28">
+      <c r="L5" s="13">
         <v>42370</v>
       </c>
       <c r="M5" t="s">
@@ -1000,13 +1011,13 @@
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="14"/>
-      <c r="B6" s="24"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
+      <c r="A6" s="25"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
       <c r="E6" s="15"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="22">
+      <c r="F6" s="10"/>
+      <c r="G6">
         <v>2</v>
       </c>
       <c r="H6" t="s">
@@ -1021,7 +1032,7 @@
       <c r="K6">
         <v>748848</v>
       </c>
-      <c r="L6" s="29" t="s">
+      <c r="L6" s="14" t="s">
         <v>73</v>
       </c>
       <c r="M6" t="s">
@@ -1029,13 +1040,13 @@
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="14"/>
-      <c r="B7" s="24"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
+      <c r="A7" s="25"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="20"/>
       <c r="E7" s="15"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="21">
+      <c r="F7" s="10"/>
+      <c r="G7" s="11">
         <v>3</v>
       </c>
       <c r="H7" t="s">
@@ -1050,7 +1061,7 @@
       <c r="K7">
         <v>748234</v>
       </c>
-      <c r="L7" s="29" t="s">
+      <c r="L7" s="14" t="s">
         <v>78</v>
       </c>
       <c r="M7" t="s">
@@ -1058,13 +1069,13 @@
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" s="14"/>
-      <c r="B8" s="24"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
+      <c r="A8" s="25"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
       <c r="E8" s="15"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="22">
+      <c r="F8" s="10"/>
+      <c r="G8">
         <v>4</v>
       </c>
       <c r="H8" t="s">
@@ -1079,7 +1090,7 @@
       <c r="K8">
         <v>748848</v>
       </c>
-      <c r="L8" s="29">
+      <c r="L8" s="14">
         <v>1132</v>
       </c>
       <c r="M8" t="s">
@@ -1087,13 +1098,13 @@
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="14"/>
-      <c r="B9" s="24"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
+      <c r="A9" s="25"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
       <c r="E9" s="15"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="21">
+      <c r="F9" s="10"/>
+      <c r="G9" s="11">
         <v>5</v>
       </c>
       <c r="H9" t="s">
@@ -1108,7 +1119,7 @@
       <c r="K9">
         <v>748848</v>
       </c>
-      <c r="L9" s="29" t="s">
+      <c r="L9" s="14" t="s">
         <v>79</v>
       </c>
       <c r="M9" t="s">
@@ -1116,13 +1127,13 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="16"/>
-      <c r="B10" s="25"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="22">
+      <c r="A10" s="26"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="10"/>
+      <c r="G10">
         <v>6</v>
       </c>
       <c r="H10" t="s">
@@ -1137,21 +1148,23 @@
       <c r="K10">
         <v>748848</v>
       </c>
-      <c r="L10" s="29" t="s">
+      <c r="L10" s="14" t="s">
         <v>74</v>
       </c>
       <c r="M10" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="21">
+    <row r="11" spans="1:13" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="11">
         <v>7</v>
       </c>
       <c r="H11" t="s">
@@ -1166,7 +1179,7 @@
       <c r="K11">
         <v>748848</v>
       </c>
-      <c r="L11" s="29">
+      <c r="L11" s="14">
         <v>1930</v>
       </c>
       <c r="M11" t="s">
@@ -1174,13 +1187,13 @@
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="10"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="22">
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12">
         <v>8</v>
       </c>
       <c r="H12" t="s">
@@ -1195,7 +1208,7 @@
       <c r="K12">
         <v>741129</v>
       </c>
-      <c r="L12" s="29" t="s">
+      <c r="L12" s="14" t="s">
         <v>80</v>
       </c>
       <c r="M12" t="s">
@@ -1203,10 +1216,10 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="G13" s="21">
+      <c r="G13" s="11">
         <v>9</v>
       </c>
       <c r="H13" t="s">
@@ -1221,7 +1234,7 @@
       <c r="K13">
         <v>741129</v>
       </c>
-      <c r="L13" s="29" t="s">
+      <c r="L13" s="14" t="s">
         <v>81</v>
       </c>
       <c r="M13" t="s">
@@ -1229,12 +1242,12 @@
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" s="27"/>
-      <c r="B14" s="27"/>
-      <c r="C14" s="27"/>
-      <c r="D14" s="27"/>
-      <c r="E14" s="27"/>
-      <c r="G14" s="22">
+      <c r="A14" s="22"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="G14">
         <v>10</v>
       </c>
       <c r="H14" t="s">
@@ -1249,7 +1262,7 @@
       <c r="K14">
         <v>741011</v>
       </c>
-      <c r="L14" s="29" t="s">
+      <c r="L14" s="14" t="s">
         <v>82</v>
       </c>
       <c r="M14" t="s">
@@ -1257,14 +1270,14 @@
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" s="27" t="s">
+      <c r="A15" s="22" t="s">
         <v>104</v>
       </c>
-      <c r="B15" s="27"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="27"/>
-      <c r="G15" s="21">
+      <c r="B15" s="22"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="G15" s="11">
         <v>11</v>
       </c>
       <c r="H15" t="s">
@@ -1279,7 +1292,7 @@
       <c r="K15">
         <v>741011</v>
       </c>
-      <c r="L15" s="29" t="s">
+      <c r="L15" s="14" t="s">
         <v>83</v>
       </c>
       <c r="M15" t="s">
@@ -1290,7 +1303,7 @@
       <c r="A16" t="s">
         <v>105</v>
       </c>
-      <c r="G16" s="22">
+      <c r="G16">
         <v>12</v>
       </c>
       <c r="H16" t="s">
@@ -1305,7 +1318,7 @@
       <c r="K16">
         <v>740899</v>
       </c>
-      <c r="L16" s="29" t="s">
+      <c r="L16" s="14" t="s">
         <v>84</v>
       </c>
       <c r="M16" t="s">
@@ -1316,7 +1329,7 @@
       <c r="A17" t="s">
         <v>106</v>
       </c>
-      <c r="G17" s="21">
+      <c r="G17" s="11">
         <v>13</v>
       </c>
       <c r="H17" t="s">
@@ -1331,7 +1344,7 @@
       <c r="K17">
         <v>740899</v>
       </c>
-      <c r="L17" s="29" t="s">
+      <c r="L17" s="14" t="s">
         <v>85</v>
       </c>
       <c r="M17" t="s">
@@ -1342,7 +1355,7 @@
       <c r="A18" t="s">
         <v>107</v>
       </c>
-      <c r="G18" s="22">
+      <c r="G18">
         <v>14</v>
       </c>
       <c r="H18" t="s">
@@ -1357,7 +1370,7 @@
       <c r="K18">
         <v>748848</v>
       </c>
-      <c r="L18" s="29">
+      <c r="L18" s="14">
         <v>15</v>
       </c>
       <c r="M18" t="s">
@@ -1368,7 +1381,7 @@
       <c r="A19" t="s">
         <v>108</v>
       </c>
-      <c r="G19" s="21">
+      <c r="G19" s="11">
         <v>15</v>
       </c>
       <c r="H19" t="s">
@@ -1383,7 +1396,7 @@
       <c r="K19">
         <v>740899</v>
       </c>
-      <c r="L19" s="29" t="s">
+      <c r="L19" s="14" t="s">
         <v>86</v>
       </c>
       <c r="M19" t="s">
@@ -1394,7 +1407,7 @@
       <c r="A20" t="s">
         <v>109</v>
       </c>
-      <c r="G20" s="22">
+      <c r="G20">
         <v>16</v>
       </c>
       <c r="H20" t="s">
@@ -1409,7 +1422,7 @@
       <c r="K20">
         <v>739429</v>
       </c>
-      <c r="L20" s="29" t="s">
+      <c r="L20" s="14" t="s">
         <v>87</v>
       </c>
       <c r="M20" t="s">
@@ -1420,7 +1433,7 @@
       <c r="A21" t="s">
         <v>110</v>
       </c>
-      <c r="G21" s="21">
+      <c r="G21" s="11">
         <v>17</v>
       </c>
       <c r="H21" t="s">
@@ -1435,7 +1448,7 @@
       <c r="K21">
         <v>748848</v>
       </c>
-      <c r="L21" s="29" t="s">
+      <c r="L21" s="14" t="s">
         <v>76</v>
       </c>
     </row>
@@ -1443,7 +1456,7 @@
       <c r="A22" t="s">
         <v>111</v>
       </c>
-      <c r="G22" s="22">
+      <c r="G22">
         <v>18</v>
       </c>
       <c r="H22" t="s">
@@ -1458,7 +1471,7 @@
       <c r="K22">
         <v>7851</v>
       </c>
-      <c r="L22" s="29" t="s">
+      <c r="L22" s="14" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1466,7 +1479,7 @@
       <c r="A23" t="s">
         <v>112</v>
       </c>
-      <c r="G23" s="21">
+      <c r="G23" s="11">
         <v>19</v>
       </c>
       <c r="H23" t="s">
@@ -1481,12 +1494,12 @@
       <c r="K23">
         <v>748848</v>
       </c>
-      <c r="L23" s="29" t="s">
+      <c r="L23" s="14" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="G24" s="22">
+      <c r="G24">
         <v>20</v>
       </c>
       <c r="H24" t="s">
@@ -1501,12 +1514,12 @@
       <c r="K24">
         <v>748846</v>
       </c>
-      <c r="L24" s="29" t="s">
+      <c r="L24" s="14" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="G25" s="21">
+      <c r="G25" s="11">
         <v>21</v>
       </c>
       <c r="H25" t="s">
@@ -1521,12 +1534,12 @@
       <c r="K25">
         <v>739429</v>
       </c>
-      <c r="L25" s="29" t="s">
+      <c r="L25" s="14" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="G26" s="22">
+      <c r="G26">
         <v>22</v>
       </c>
       <c r="H26" t="s">
@@ -1541,12 +1554,12 @@
       <c r="K26">
         <v>739429</v>
       </c>
-      <c r="L26" s="29" t="s">
+      <c r="L26" s="14" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="G27" s="21">
+      <c r="G27" s="11">
         <v>23</v>
       </c>
       <c r="H27" t="s">
@@ -1561,12 +1574,12 @@
       <c r="K27">
         <v>748848</v>
       </c>
-      <c r="L27" s="29" t="s">
+      <c r="L27" s="14" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="G28" s="22">
+      <c r="G28">
         <v>24</v>
       </c>
       <c r="H28" t="s">
@@ -1581,12 +1594,12 @@
       <c r="K28">
         <v>99999</v>
       </c>
-      <c r="L28" s="29" t="s">
+      <c r="L28" s="14" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="G29" s="21">
+      <c r="G29" s="11">
         <v>25</v>
       </c>
       <c r="H29" t="s">
@@ -1601,12 +1614,12 @@
       <c r="K29">
         <v>99999</v>
       </c>
-      <c r="L29" s="29" t="s">
+      <c r="L29" s="14" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="G30" s="22">
+      <c r="G30">
         <v>26</v>
       </c>
       <c r="H30" t="s">
@@ -1621,12 +1634,12 @@
       <c r="K30">
         <v>99999</v>
       </c>
-      <c r="L30" s="29" t="s">
+      <c r="L30" s="14" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="G31" s="21">
+      <c r="G31" s="11">
         <v>27</v>
       </c>
       <c r="H31" t="s">
@@ -1641,12 +1654,12 @@
       <c r="K31">
         <v>99999</v>
       </c>
-      <c r="L31" s="29" t="s">
+      <c r="L31" s="14" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="G32" s="22">
+      <c r="G32">
         <v>28</v>
       </c>
       <c r="H32" t="s">
@@ -1661,12 +1674,12 @@
       <c r="K32">
         <v>99999</v>
       </c>
-      <c r="L32" s="29" t="s">
+      <c r="L32" s="14" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="33" spans="7:13" x14ac:dyDescent="0.25">
-      <c r="G33" s="21">
+      <c r="G33" s="11">
         <v>29</v>
       </c>
       <c r="H33" t="s">
@@ -1681,7 +1694,7 @@
       <c r="K33">
         <v>0</v>
       </c>
-      <c r="L33" s="29" t="s">
+      <c r="L33" s="14" t="s">
         <v>77</v>
       </c>
       <c r="M33" t="s">
@@ -1690,18 +1703,21 @@
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A5:A10"/>
     <mergeCell ref="E5:E10"/>
     <mergeCell ref="B5:B10"/>
     <mergeCell ref="C5:C10"/>
     <mergeCell ref="D5:D10"/>
     <mergeCell ref="A14:E14"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:A10"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="D5" r:id="rId1" xr:uid="{A4B529EF-448E-45CC-AE68-AE907E4CD54C}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>